<commit_message>
NOM.OL CR:c|high|double. + Excel + D&A
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/NOM.OL.xlsx
+++ b/data/obx_xlsx/NOM.OL.xlsx
@@ -2517,10 +2517,22 @@
       <c r="B27" s="19">
         <v>107.76</v>
       </c>
-      <c r="C27" s="15"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
+      <c r="C27" s="14">
+        <f t="shared" ref="C27:F27" si="1">SUM(C28:C30)</f>
+        <v>5.45</v>
+      </c>
+      <c r="D27" s="14">
+        <f t="shared" si="1"/>
+        <v>0.7</v>
+      </c>
+      <c r="E27" s="14">
+        <f t="shared" si="1"/>
+        <v>0.32</v>
+      </c>
+      <c r="F27" s="14">
+        <f t="shared" si="1"/>
+        <v>0.28</v>
+      </c>
       <c r="G27" s="14">
         <v>0.24</v>
       </c>

</xml_diff>